<commit_message>
fix(demo): normalize all Excel and CSV import templates to clean English to prevent font encoding issues
</commit_message>
<xml_diff>
--- a/Report/Demo_Assessment_Import_Scores.xlsx
+++ b/Report/Demo_Assessment_Import_Scores.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nhập điểm" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assessment Scores" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -28,13 +28,13 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="001E293B"/>
+      <color rgb="001F497D"/>
       <sz val="13"/>
     </font>
     <font>
       <name val="Calibri"/>
       <i val="1"/>
-      <color rgb="00475569"/>
+      <color rgb="00595959"/>
       <sz val="10"/>
     </font>
     <font>
@@ -45,10 +45,10 @@
     </font>
     <font>
       <name val="Calibri"/>
-      <sz val="10"/>
+      <sz val="11"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -57,14 +57,20 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F1F5F9"/>
-        <bgColor rgb="00F1F5F9"/>
+        <fgColor rgb="00DCE6F1"/>
+        <bgColor rgb="00DCE6F1"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001E293B"/>
-        <bgColor rgb="001E293B"/>
+        <fgColor rgb="00F2F2F2"/>
+        <bgColor rgb="00F2F2F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004F81BD"/>
+        <bgColor rgb="004F81BD"/>
       </patternFill>
     </fill>
   </fills>
@@ -78,16 +84,16 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00CBD5E1"/>
+        <color rgb="00D9D9D9"/>
       </left>
       <right style="thin">
-        <color rgb="00CBD5E1"/>
+        <color rgb="00D9D9D9"/>
       </right>
       <top style="thin">
-        <color rgb="00CBD5E1"/>
+        <color rgb="00D9D9D9"/>
       </top>
       <bottom style="thin">
-        <color rgb="00CBD5E1"/>
+        <color rgb="00D9D9D9"/>
       </bottom>
     </border>
   </borders>
@@ -96,20 +102,20 @@
   </cellStyleXfs>
   <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -479,18 +485,18 @@
   <dimension ref="A1:F7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="19" customWidth="1" min="1" max="1"/>
+    <col width="80" customWidth="1" min="1" max="1"/>
     <col width="49" customWidth="1" min="2" max="2"/>
     <col width="20" customWidth="1" min="3" max="3"/>
     <col width="19" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="42" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="45" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>BẢNG NHẬP ĐIỂM - Final Exam (Theory) - Môn: Aviation Regulations</t>
+          <t>ASSESSMENT SCORE ENTRY - Final Exam (Theory) - Subject: Aviation Regulations</t>
         </is>
       </c>
     </row>
@@ -522,11 +528,11 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Môn: Aviation Regulations</t>
+          <t>Subject: Aviation Regulations</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="24" customHeight="1">
+    <row r="3" ht="25" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
           <t>AccountId</t>
@@ -534,12 +540,12 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Họ và tên</t>
+          <t>Full Name</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>Mã học viên</t>
+          <t>Student Code</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
@@ -549,12 +555,12 @@
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>Điểm số (0-100)*</t>
+          <t>Score (0-100)*</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>Ghi chú</t>
+          <t>Remarks</t>
         </is>
       </c>
     </row>
@@ -562,7 +568,7 @@
       <c r="A4" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>Jane Student</t>
         </is>
@@ -575,12 +581,12 @@
       <c r="D4" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="E4" s="4" t="n">
+      <c r="E4" s="5" t="n">
         <v>88.5</v>
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>Đạt yêu cầu - Kỹ năng nắm vững</t>
+          <t>Pass - Solid technical knowledge</t>
         </is>
       </c>
     </row>
@@ -588,7 +594,7 @@
       <c r="A5" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="B5" s="5" t="inlineStr">
+      <c r="B5" s="4" t="inlineStr">
         <is>
           <t>Student 2</t>
         </is>
@@ -601,12 +607,12 @@
       <c r="D5" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="E5" s="4" t="n">
+      <c r="E5" s="5" t="n">
         <v>92</v>
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>Xuất sắc - Hoàn thành xuất sắc bài thi</t>
+          <t>Distinction - Excellent exam performance</t>
         </is>
       </c>
     </row>
@@ -614,7 +620,7 @@
       <c r="A6" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="B6" s="5" t="inlineStr">
+      <c r="B6" s="4" t="inlineStr">
         <is>
           <t>Student 3</t>
         </is>
@@ -627,12 +633,12 @@
       <c r="D6" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="E6" s="4" t="n">
+      <c r="E6" s="5" t="n">
         <v>75</v>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>Đạt yêu cầu - Cần rà soát thêm quy chế</t>
+          <t>Pass - Review flight regulations required</t>
         </is>
       </c>
     </row>
@@ -640,7 +646,7 @@
       <c r="A7" s="4" t="n">
         <v>11</v>
       </c>
-      <c r="B7" s="5" t="inlineStr">
+      <c r="B7" s="4" t="inlineStr">
         <is>
           <t>Student 4</t>
         </is>
@@ -653,12 +659,12 @@
       <c r="D7" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="E7" s="4" t="n">
+      <c r="E7" s="5" t="n">
         <v>84</v>
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>Đạt yêu cầu - Thao tác tốt</t>
+          <t>Pass - Good practical procedures</t>
         </is>
       </c>
     </row>

</xml_diff>